<commit_message>
Refactoring code + redownloading excel sheet
</commit_message>
<xml_diff>
--- a/Sprint_Report/TeamEReport.xlsx
+++ b/Sprint_Report/TeamEReport.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="211">
   <si>
     <t>Initials</t>
   </si>
@@ -368,6 +368,21 @@
     <t>Sibling Spacing (8 months apart)</t>
   </si>
   <si>
+    <t xml:space="preserve">Completing Stories on Time: All 6 planned user stories were implemented and verified against the test GEDCOM file by the sprint deadline. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good Communication: Team members met for weekly zoom meeting and communicated throughout the week through messaging to divide GEDCOM user stories and resolve issues. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relying on a single testfile: Team members will create a new testfile for each user story to cover normal cases, edge cases and boundary conditions. </t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Multiple Births &lt;= 5</t>
+  </si>
+  <si>
     <t>Story Description</t>
   </si>
   <si>
@@ -459,9 +474,6 @@
   </si>
   <si>
     <t>Siblings should not marry one another</t>
-  </si>
-  <si>
-    <t>First cousins should not marry one another</t>
   </si>
   <si>
     <t>Aunts and uncles</t>
@@ -651,9 +663,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="m/d"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="mm/dd"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -726,7 +739,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -769,6 +782,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -814,11 +830,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1113012086"/>
-        <c:axId val="993125955"/>
+        <c:axId val="1411270868"/>
+        <c:axId val="301430367"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1113012086"/>
+        <c:axId val="1411270868"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -870,10 +886,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="993125955"/>
+        <c:crossAx val="301430367"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="993125955"/>
+        <c:axId val="301430367"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -937,7 +953,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1113012086"/>
+        <c:crossAx val="1411270868"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -978,11 +994,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="949758386"/>
-        <c:axId val="1096522443"/>
+        <c:axId val="1397272643"/>
+        <c:axId val="249227662"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="949758386"/>
+        <c:axId val="1397272643"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1034,10 +1050,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1096522443"/>
+        <c:crossAx val="249227662"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1096522443"/>
+        <c:axId val="249227662"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1101,7 +1117,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="949758386"/>
+        <c:crossAx val="1397272643"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -3287,10 +3303,13 @@
         <v>10</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
+      <c r="A12" s="7">
+        <v>3.0</v>
+      </c>
       <c r="B12" s="2" t="s">
         <v>51</v>
       </c>
@@ -3302,6 +3321,9 @@
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
+      <c r="A13" s="7">
+        <v>3.0</v>
+      </c>
       <c r="B13" s="2" t="s">
         <v>53</v>
       </c>
@@ -3326,10 +3348,13 @@
         <v>15</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
+      <c r="A15" s="7">
+        <v>3.0</v>
+      </c>
       <c r="B15" s="2" t="s">
         <v>57</v>
       </c>
@@ -3354,10 +3379,13 @@
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" ht="12.75" customHeight="1">
+      <c r="A17" s="7">
+        <v>3.0</v>
+      </c>
       <c r="B17" s="2" t="s">
         <v>61</v>
       </c>
@@ -3425,7 +3453,7 @@
         <v>10</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" ht="12.75" customHeight="1">
@@ -8702,7 +8730,8 @@
         <v>580.0</v>
       </c>
       <c r="F3" s="10">
-        <v>73.9</v>
+        <f t="shared" ref="F3:F6" si="1">(D3-D2)/E3*60</f>
+        <v>69.51724138</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -8715,16 +8744,46 @@
       <c r="C4" s="7">
         <v>6.0</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="F4" s="10"/>
+      <c r="D4" s="7">
+        <v>395.0</v>
+      </c>
+      <c r="E4" s="7">
+        <v>262.0</v>
+      </c>
+      <c r="F4" s="10">
+        <f t="shared" si="1"/>
+        <v>-63.4351145</v>
+      </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="F5" s="10"/>
+      <c r="A5" s="17">
+        <v>46208.0</v>
+      </c>
+      <c r="B5" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="C5" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="F5" s="10" t="str">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="F6" s="10"/>
+      <c r="A6" s="17">
+        <v>46215.0</v>
+      </c>
+      <c r="B6" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="C6" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="F6" s="10" t="str">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="9"/>
@@ -16959,7 +17018,9 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="10.78"/>
+    <col customWidth="1" min="1" max="1" width="10.78"/>
+    <col customWidth="1" min="2" max="2" width="28.56"/>
+    <col customWidth="1" min="3" max="26" width="10.78"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
@@ -17002,13 +17063,22 @@
         <v>5</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E2" s="7">
         <v>10.0</v>
       </c>
       <c r="F2" s="7">
         <v>60.0</v>
+      </c>
+      <c r="G2" s="7">
+        <v>27.0</v>
+      </c>
+      <c r="H2" s="7">
+        <v>36.0</v>
+      </c>
+      <c r="I2" s="23">
+        <v>46199.0</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1">
@@ -17022,13 +17092,22 @@
         <v>5</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E3" s="7">
         <v>10.0</v>
       </c>
       <c r="F3" s="7">
         <v>60.0</v>
+      </c>
+      <c r="G3" s="7">
+        <v>70.0</v>
+      </c>
+      <c r="H3" s="7">
+        <v>75.0</v>
+      </c>
+      <c r="I3" s="23">
+        <v>46200.0</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -17042,13 +17121,22 @@
         <v>10</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E4" s="7">
         <v>15.0</v>
       </c>
       <c r="F4" s="7">
         <v>45.0</v>
+      </c>
+      <c r="G4" s="7">
+        <v>22.0</v>
+      </c>
+      <c r="H4" s="7">
+        <v>39.0</v>
+      </c>
+      <c r="I4" s="23">
+        <v>46199.0</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
@@ -17062,13 +17150,22 @@
         <v>10</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E5" s="7">
         <v>15.0</v>
       </c>
       <c r="F5" s="7">
         <v>45.0</v>
+      </c>
+      <c r="G5" s="7">
+        <v>25.0</v>
+      </c>
+      <c r="H5" s="7">
+        <v>27.0</v>
+      </c>
+      <c r="I5" s="23">
+        <v>46199.0</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
@@ -17082,13 +17179,22 @@
         <v>15</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E6" s="7">
         <v>20.0</v>
       </c>
       <c r="F6" s="7">
         <v>45.0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>130.0</v>
+      </c>
+      <c r="H6" s="7">
+        <v>40.0</v>
+      </c>
+      <c r="I6" s="23">
+        <v>46199.0</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1">
@@ -17102,13 +17208,22 @@
         <v>15</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="E7" s="7">
         <v>20.0</v>
       </c>
       <c r="F7" s="7">
         <v>45.0</v>
+      </c>
+      <c r="G7" s="7">
+        <v>121.0</v>
+      </c>
+      <c r="H7" s="7">
+        <v>45.0</v>
+      </c>
+      <c r="I7" s="23">
+        <v>46199.0</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1"/>
@@ -17117,15 +17232,45 @@
     <row r="11" ht="12.75" customHeight="1"/>
     <row r="12" ht="12.75" customHeight="1"/>
     <row r="13" ht="12.75" customHeight="1"/>
-    <row r="14" ht="12.75" customHeight="1"/>
-    <row r="15" ht="12.75" customHeight="1"/>
-    <row r="16" ht="12.75" customHeight="1"/>
-    <row r="17" ht="12.75" customHeight="1"/>
-    <row r="18" ht="12.75" customHeight="1"/>
-    <row r="19" ht="12.75" customHeight="1"/>
-    <row r="20" ht="12.75" customHeight="1"/>
-    <row r="21" ht="12.75" customHeight="1"/>
-    <row r="22" ht="12.75" customHeight="1"/>
+    <row r="14" ht="12.75" customHeight="1">
+      <c r="B14" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" ht="12.75" customHeight="1">
+      <c r="B15" s="22"/>
+    </row>
+    <row r="16" ht="12.75" customHeight="1">
+      <c r="B16" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" ht="62.25" customHeight="1">
+      <c r="B17" s="21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" ht="63.75" customHeight="1">
+      <c r="B18" s="21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" ht="12.75" customHeight="1">
+      <c r="B19" s="4"/>
+    </row>
+    <row r="20" ht="12.75" customHeight="1">
+      <c r="B20" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" ht="61.5" customHeight="1">
+      <c r="B21" s="21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" ht="12.75" customHeight="1">
+      <c r="B22" s="7"/>
+    </row>
     <row r="23" ht="12.75" customHeight="1"/>
     <row r="24" ht="12.75" customHeight="1"/>
     <row r="25" ht="12.75" customHeight="1"/>
@@ -18119,7 +18264,9 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="10.78"/>
+    <col customWidth="1" min="1" max="1" width="10.78"/>
+    <col customWidth="1" min="2" max="2" width="19.67"/>
+    <col customWidth="1" min="3" max="26" width="10.78"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
@@ -18151,10 +18298,86 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" ht="12.75" customHeight="1"/>
-    <row r="3" ht="12.75" customHeight="1"/>
-    <row r="4" ht="12.75" customHeight="1"/>
-    <row r="5" ht="12.75" customHeight="1"/>
+    <row r="2" ht="12.75" customHeight="1">
+      <c r="A2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="F2" s="7">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="3" ht="12.75" customHeight="1">
+      <c r="A3" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E3" s="7">
+        <v>15.0</v>
+      </c>
+      <c r="F3" s="7">
+        <v>45.0</v>
+      </c>
+    </row>
+    <row r="4" ht="12.75" customHeight="1">
+      <c r="A4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="7">
+        <v>25.0</v>
+      </c>
+      <c r="F4" s="7">
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="5" ht="12.75" customHeight="1">
+      <c r="A5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E5" s="7">
+        <v>20.0</v>
+      </c>
+      <c r="F5" s="7">
+        <v>45.0</v>
+      </c>
+    </row>
     <row r="6" ht="12.75" customHeight="1"/>
     <row r="7" ht="12.75" customHeight="1"/>
     <row r="8" ht="12.75" customHeight="1"/>
@@ -20225,7 +20448,7 @@
         <v>24</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -20258,8 +20481,8 @@
       <c r="B2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="23" t="s">
-        <v>115</v>
+      <c r="C2" s="24" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1">
@@ -20267,10 +20490,10 @@
         <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>117</v>
+        <v>121</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -20280,19 +20503,19 @@
       <c r="B4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>118</v>
+      <c r="C4" s="24" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>121</v>
+        <v>125</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
@@ -20300,10 +20523,10 @@
         <v>37</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>123</v>
+        <v>127</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1">
@@ -20311,10 +20534,10 @@
         <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>125</v>
+        <v>129</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
@@ -20322,10 +20545,10 @@
         <v>42</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>127</v>
+        <v>131</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
@@ -20333,10 +20556,10 @@
         <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>129</v>
+        <v>133</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
@@ -20344,10 +20567,10 @@
         <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>131</v>
+        <v>135</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
@@ -20357,8 +20580,8 @@
       <c r="B11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>132</v>
+      <c r="C11" s="24" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
@@ -20368,8 +20591,8 @@
       <c r="B12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>133</v>
+      <c r="C12" s="24" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
@@ -20377,10 +20600,10 @@
         <v>53</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>135</v>
+        <v>139</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1">
@@ -20388,10 +20611,10 @@
         <v>55</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>137</v>
+        <v>141</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
@@ -20401,8 +20624,8 @@
       <c r="B15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="23" t="s">
-        <v>138</v>
+      <c r="C15" s="24" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
@@ -20410,10 +20633,10 @@
         <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>140</v>
+        <v>144</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="17" ht="12.75" customHeight="1">
@@ -20421,10 +20644,10 @@
         <v>61</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>142</v>
+        <v>146</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="18" ht="12.75" customHeight="1">
@@ -20434,8 +20657,8 @@
       <c r="B18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>143</v>
+      <c r="C18" s="24" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="19" ht="12.75" customHeight="1">
@@ -20445,8 +20668,8 @@
       <c r="B19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="23" t="s">
-        <v>144</v>
+      <c r="C19" s="24" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="20" ht="12.75" customHeight="1">
@@ -20456,18 +20679,16 @@
       <c r="B20" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="23" t="s">
-        <v>145</v>
-      </c>
+      <c r="C20" s="24"/>
     </row>
     <row r="21" ht="12.75" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C21" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="24" t="s">
         <v>64</v>
       </c>
     </row>
@@ -20476,10 +20697,10 @@
         <v>71</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>148</v>
+        <v>151</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="23" ht="12.75" customHeight="1">
@@ -20489,8 +20710,8 @@
       <c r="B23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="23" t="s">
-        <v>149</v>
+      <c r="C23" s="24" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="24" ht="12.75" customHeight="1">
@@ -20498,21 +20719,21 @@
         <v>75</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>151</v>
+        <v>154</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="25" ht="12.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>154</v>
+        <v>157</v>
+      </c>
+      <c r="C25" s="24" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="26" ht="12.75" customHeight="1">
@@ -20520,197 +20741,197 @@
         <v>79</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>156</v>
+        <v>159</v>
+      </c>
+      <c r="C26" s="24" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="27" ht="12.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>159</v>
+        <v>162</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>162</v>
+        <v>165</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>165</v>
+        <v>168</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>168</v>
+        <v>171</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="C31" s="23" t="s">
-        <v>171</v>
+        <v>174</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>177</v>
+        <v>180</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C34" s="23" t="s">
-        <v>180</v>
+        <v>183</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C35" s="23" t="s">
-        <v>183</v>
+        <v>186</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>186</v>
+        <v>189</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>189</v>
+        <v>192</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="C38" s="23" t="s">
-        <v>192</v>
+        <v>195</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C39" s="23" t="s">
-        <v>195</v>
+        <v>198</v>
+      </c>
+      <c r="C39" s="24" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>198</v>
+        <v>201</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>201</v>
+        <v>204</v>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>204</v>
+        <v>207</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C43" s="23" t="s">
-        <v>206</v>
+      <c r="C43" s="24" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="44" ht="12.75" customHeight="1">

</xml_diff>

<commit_message>
Downloaded updated team report
</commit_message>
<xml_diff>
--- a/Sprint_Report/TeamEReport.xlsx
+++ b/Sprint_Report/TeamEReport.xlsx
@@ -831,11 +831,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="296122275"/>
-        <c:axId val="1497330205"/>
+        <c:axId val="688225807"/>
+        <c:axId val="858514025"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="296122275"/>
+        <c:axId val="688225807"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -887,10 +887,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1497330205"/>
+        <c:crossAx val="858514025"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1497330205"/>
+        <c:axId val="858514025"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -954,7 +954,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="296122275"/>
+        <c:crossAx val="688225807"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -995,11 +995,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="202678943"/>
-        <c:axId val="446950256"/>
+        <c:axId val="859471244"/>
+        <c:axId val="926504897"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="202678943"/>
+        <c:axId val="859471244"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1051,10 +1051,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="446950256"/>
+        <c:crossAx val="926504897"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="446950256"/>
+        <c:axId val="926504897"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1118,7 +1118,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="202678943"/>
+        <c:crossAx val="859471244"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -18448,7 +18448,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="E5" s="8">
         <v>20.0</v>
@@ -18456,7 +18456,15 @@
       <c r="F5" s="8">
         <v>45.0</v>
       </c>
-      <c r="I5" s="24"/>
+      <c r="G5" s="8">
+        <v>30.0</v>
+      </c>
+      <c r="H5" s="8">
+        <v>40.0</v>
+      </c>
+      <c r="I5" s="24">
+        <v>46217.0</v>
+      </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="8" t="s">

</xml_diff>